<commit_message>
update the analysis to render better and make word and pdfs
</commit_message>
<xml_diff>
--- a/data/raw/NCE_data.xlsx
+++ b/data/raw/NCE_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://waikatouniversitynz-my.sharepoint.com/personal/or81_students_waikato_ac_nz/Documents/Documents/PhD/01_thesis_chapters/05_fear_study/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="8_{1C509BC5-B9CD-4355-A94E-B3E32C99D6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{003AD1E5-8066-4073-A0FE-EAFF5DE9D967}"/>
+  <xr:revisionPtr revIDLastSave="145" documentId="8_{1C509BC5-B9CD-4355-A94E-B3E32C99D6B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A37559C7-E1B4-4771-8AD6-26F106EB4C95}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{884ED942-72D7-478A-91F6-B92A4F060477}"/>
+    <workbookView minimized="1" xWindow="58395" yWindow="3450" windowWidth="7500" windowHeight="6000" xr2:uid="{884ED942-72D7-478A-91F6-B92A4F060477}"/>
   </bookViews>
   <sheets>
     <sheet name="NCE_exp" sheetId="2" r:id="rId1"/>
@@ -805,7 +805,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -823,6 +823,7 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4774,34 +4775,35 @@
       <c r="AY19" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="BA19">
+      <c r="BA19" s="17">
         <v>58</v>
       </c>
-      <c r="BB19">
+      <c r="BB19" s="17">
         <v>58</v>
       </c>
-      <c r="BD19">
-        <v>2</v>
-      </c>
-      <c r="BE19" t="s">
-        <v>1</v>
-      </c>
-      <c r="BF19" t="s">
-        <v>1</v>
-      </c>
-      <c r="BG19">
+      <c r="BC19" s="17"/>
+      <c r="BD19" s="17">
+        <v>2</v>
+      </c>
+      <c r="BE19" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="BF19" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="BG19" s="17">
         <v>26.88</v>
       </c>
-      <c r="BH19">
+      <c r="BH19" s="17">
         <v>13</v>
       </c>
-      <c r="BI19">
+      <c r="BI19" s="17">
         <v>8</v>
       </c>
-      <c r="BJ19">
+      <c r="BJ19" s="17">
         <v>0</v>
       </c>
-      <c r="BK19">
+      <c r="BK19" s="17">
         <v>2</v>
       </c>
       <c r="BR19" s="2"/>
@@ -11506,7 +11508,7 @@
         <v>9</v>
       </c>
       <c r="BA56">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="BB56">
         <v>75</v>
@@ -12773,37 +12775,37 @@
       <c r="AY63" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="BA63">
+      <c r="BA63" s="17">
         <v>102</v>
       </c>
-      <c r="BB63">
+      <c r="BB63" s="17">
         <v>102</v>
       </c>
-      <c r="BC63">
+      <c r="BC63" s="17">
         <v>58</v>
       </c>
-      <c r="BD63">
+      <c r="BD63" s="17">
         <v>14</v>
       </c>
-      <c r="BE63" t="s">
-        <v>1</v>
-      </c>
-      <c r="BF63" t="s">
-        <v>1</v>
-      </c>
-      <c r="BG63">
+      <c r="BE63" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="BF63" s="17" t="s">
+        <v>1</v>
+      </c>
+      <c r="BG63" s="17">
         <v>26.87</v>
       </c>
-      <c r="BH63">
+      <c r="BH63" s="17">
         <v>11</v>
       </c>
-      <c r="BI63">
+      <c r="BI63" s="17">
         <v>7</v>
       </c>
-      <c r="BJ63">
-        <v>2</v>
-      </c>
-      <c r="BK63">
+      <c r="BJ63" s="17">
+        <v>2</v>
+      </c>
+      <c r="BK63" s="17">
         <v>2</v>
       </c>
       <c r="BR63" s="2"/>

</xml_diff>